<commit_message>
Add Extender. Add few Mux signals. Minor fixes in Green Card
</commit_message>
<xml_diff>
--- a/opcode to control bits.xlsx
+++ b/opcode to control bits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrai\Documents\SC8bCPU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA8D103-272E-4016-BFFA-58C0C0F31500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5A3259-C6E8-4060-9270-6DA0E14B4B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4797" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4803" uniqueCount="188">
   <si>
     <t>Instruction</t>
   </si>
@@ -606,6 +606,12 @@
   <si>
     <t>DIVDU</t>
   </si>
+  <si>
+    <t>SIGNED</t>
+  </si>
+  <si>
+    <t>PC_IN[1:0]</t>
+  </si>
 </sst>
 </file>
 
@@ -655,11 +661,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -30603,7 +30608,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D896E85-B550-461A-BB89-06512C5EBBCD}">
-  <dimension ref="A1:U62"/>
+  <dimension ref="A1:W62"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.46484375" style="1" bestFit="1" customWidth="1"/>
@@ -30627,9 +30632,10 @@
     <col min="19" max="19" width="15.1328125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="8.9296875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -30663,13 +30669,13 @@
       <c r="K1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="1" t="s">
         <v>175</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="1" t="s">
         <v>176</v>
       </c>
       <c r="O1" s="1" t="s">
@@ -30693,8 +30699,14 @@
       <c r="U1" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>24</v>
       </c>
@@ -30705,7 +30717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
@@ -30713,7 +30725,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>48</v>
       </c>
@@ -30732,14 +30744,14 @@
       <c r="M4" t="s">
         <v>126</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>126</v>
       </c>
       <c r="U4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>92</v>
       </c>
@@ -30755,14 +30767,14 @@
       <c r="M5" t="s">
         <v>126</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>126</v>
       </c>
       <c r="U5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>50</v>
       </c>
@@ -30781,14 +30793,14 @@
       <c r="M6" t="s">
         <v>126</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="P6" t="s">
         <v>119</v>
       </c>
       <c r="U6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>97</v>
       </c>
@@ -30814,16 +30826,16 @@
         <v>119</v>
       </c>
       <c r="P7" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q7" t="s">
         <v>126</v>
       </c>
-      <c r="Q7" t="s">
-        <v>119</v>
-      </c>
       <c r="U7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>138</v>
       </c>
@@ -30843,16 +30855,16 @@
         <v>180</v>
       </c>
       <c r="P8" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q8" t="s">
         <v>126</v>
       </c>
-      <c r="Q8" t="s">
-        <v>119</v>
-      </c>
       <c r="U8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>111</v>
       </c>
@@ -30874,11 +30886,14 @@
       <c r="M9" t="s">
         <v>126</v>
       </c>
+      <c r="P9" t="s">
+        <v>119</v>
+      </c>
       <c r="U9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>95</v>
       </c>
@@ -30901,16 +30916,16 @@
         <v>126</v>
       </c>
       <c r="P10" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q10" t="s">
         <v>126</v>
       </c>
-      <c r="Q10" t="s">
-        <v>119</v>
-      </c>
       <c r="U10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>96</v>
       </c>
@@ -30936,16 +30951,16 @@
         <v>126</v>
       </c>
       <c r="P11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q11" t="s">
         <v>126</v>
       </c>
-      <c r="Q11" t="s">
-        <v>119</v>
-      </c>
       <c r="U11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>139</v>
       </c>
@@ -30955,7 +30970,7 @@
       <c r="C12" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P12" t="s">
+      <c r="Q12" t="s">
         <v>126</v>
       </c>
       <c r="T12">
@@ -30964,8 +30979,11 @@
       <c r="U12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>140</v>
       </c>
@@ -30984,7 +31002,7 @@
       <c r="O13" t="s">
         <v>119</v>
       </c>
-      <c r="P13" t="s">
+      <c r="Q13" t="s">
         <v>126</v>
       </c>
       <c r="T13">
@@ -30993,8 +31011,11 @@
       <c r="U13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>141</v>
       </c>
@@ -31004,7 +31025,7 @@
       <c r="C14" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P14" t="s">
+      <c r="Q14" t="s">
         <v>126</v>
       </c>
       <c r="T14" t="s">
@@ -31013,8 +31034,11 @@
       <c r="U14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>142</v>
       </c>
@@ -31024,7 +31048,7 @@
       <c r="C15" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P15" t="s">
+      <c r="Q15" t="s">
         <v>126</v>
       </c>
       <c r="T15" t="s">
@@ -31033,8 +31057,11 @@
       <c r="U15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>144</v>
       </c>
@@ -31044,7 +31071,7 @@
       <c r="C16" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P16" t="s">
+      <c r="Q16" t="s">
         <v>126</v>
       </c>
       <c r="T16" t="s">
@@ -31053,8 +31080,11 @@
       <c r="U16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>143</v>
       </c>
@@ -31064,7 +31094,7 @@
       <c r="C17" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P17" t="s">
+      <c r="Q17" t="s">
         <v>126</v>
       </c>
       <c r="T17" t="s">
@@ -31073,8 +31103,11 @@
       <c r="U17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
@@ -31093,8 +31126,11 @@
       <c r="U18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>145</v>
       </c>
@@ -31114,7 +31150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>146</v>
       </c>
@@ -31133,11 +31169,20 @@
       <c r="M20" t="s">
         <v>153</v>
       </c>
+      <c r="P20" t="s">
+        <v>126</v>
+      </c>
+      <c r="S20">
+        <v>3</v>
+      </c>
       <c r="U20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>147</v>
       </c>
@@ -31156,11 +31201,20 @@
       <c r="M21" t="s">
         <v>153</v>
       </c>
+      <c r="P21" t="s">
+        <v>126</v>
+      </c>
+      <c r="S21">
+        <v>1</v>
+      </c>
       <c r="U21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>148</v>
       </c>
@@ -31179,11 +31233,20 @@
       <c r="M22" t="s">
         <v>153</v>
       </c>
+      <c r="P22" t="s">
+        <v>126</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
       <c r="U22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>149</v>
       </c>
@@ -31196,14 +31259,20 @@
       <c r="D23" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P23" t="s">
+      <c r="Q23" t="s">
         <v>153</v>
       </c>
+      <c r="S23">
+        <v>3</v>
+      </c>
       <c r="U23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>150</v>
       </c>
@@ -31216,14 +31285,20 @@
       <c r="D24" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P24" t="s">
+      <c r="Q24" t="s">
         <v>153</v>
       </c>
+      <c r="S24">
+        <v>1</v>
+      </c>
       <c r="U24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>151</v>
       </c>
@@ -31236,14 +31311,20 @@
       <c r="D25" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="P25" t="s">
+      <c r="Q25" t="s">
         <v>153</v>
       </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
       <c r="U25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>107</v>
       </c>
@@ -31272,7 +31353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>63</v>
       </c>
@@ -31285,8 +31366,14 @@
       <c r="U27">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V27">
+        <v>1</v>
+      </c>
+      <c r="W27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>66</v>
       </c>
@@ -31299,8 +31386,14 @@
       <c r="U28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V28">
+        <v>1</v>
+      </c>
+      <c r="W28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>87</v>
       </c>
@@ -31313,8 +31406,14 @@
       <c r="U29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V29">
+        <v>1</v>
+      </c>
+      <c r="W29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>152</v>
       </c>
@@ -31334,7 +31433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>101</v>
       </c>
@@ -31381,7 +31480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>95</v>
       </c>
@@ -31996,6 +32095,9 @@
       <c r="H45" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="I45">
+        <v>1</v>
+      </c>
       <c r="J45">
         <v>5</v>
       </c>
@@ -32040,6 +32142,9 @@
       <c r="H46" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="I46">
+        <v>1</v>
+      </c>
       <c r="J46">
         <v>5</v>
       </c>
@@ -32147,7 +32252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A49" s="1" t="s">
         <v>100</v>
       </c>
@@ -32172,6 +32277,9 @@
       <c r="H49" s="2" t="s">
         <v>136</v>
       </c>
+      <c r="I49">
+        <v>1</v>
+      </c>
       <c r="J49">
         <v>7</v>
       </c>
@@ -32191,7 +32299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A50" s="1" t="s">
         <v>158</v>
       </c>
@@ -32216,6 +32324,9 @@
       <c r="H50" s="2" t="s">
         <v>137</v>
       </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
       <c r="J50">
         <v>7</v>
       </c>
@@ -32235,7 +32346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A51" s="1" t="s">
         <v>159</v>
       </c>
@@ -32260,9 +32371,6 @@
       <c r="H51" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="I51">
-        <v>1</v>
-      </c>
       <c r="K51" s="1" t="s">
         <v>183</v>
       </c>
@@ -32290,8 +32398,11 @@
       <c r="U51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A52" s="1" t="s">
         <v>160</v>
       </c>
@@ -32316,9 +32427,6 @@
       <c r="H52" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="I52">
-        <v>1</v>
-      </c>
       <c r="K52" s="1" t="s">
         <v>183</v>
       </c>
@@ -32343,8 +32451,11 @@
       <c r="U52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A53" s="1" t="s">
         <v>161</v>
       </c>
@@ -32397,7 +32508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A54" s="1" t="s">
         <v>162</v>
       </c>
@@ -32447,7 +32558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A55" s="1" t="s">
         <v>184</v>
       </c>
@@ -32472,9 +32583,6 @@
       <c r="H55" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="I55">
-        <v>1</v>
-      </c>
       <c r="K55" s="1" t="s">
         <v>182</v>
       </c>
@@ -32502,8 +32610,11 @@
       <c r="U55">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A56" s="1" t="s">
         <v>163</v>
       </c>
@@ -32528,9 +32639,6 @@
       <c r="H56" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="I56">
-        <v>1</v>
-      </c>
       <c r="K56" s="1" t="s">
         <v>182</v>
       </c>
@@ -32555,8 +32663,11 @@
       <c r="U56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="V56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A57" s="1" t="s">
         <v>185</v>
       </c>
@@ -32609,7 +32720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A58" s="1" t="s">
         <v>164</v>
       </c>
@@ -32659,7 +32770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A59" s="1" t="s">
         <v>167</v>
       </c>
@@ -32687,8 +32798,11 @@
       <c r="U59">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A60" s="1" t="s">
         <v>168</v>
       </c>
@@ -32716,8 +32830,11 @@
       <c r="U60">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="W60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A61" s="1" t="s">
         <v>58</v>
       </c>
@@ -32758,7 +32875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A62" s="1" t="s">
         <v>169</v>
       </c>

</xml_diff>

<commit_message>
Finish control signal addition. Change instruction field positions
</commit_message>
<xml_diff>
--- a/opcode to control bits.xlsx
+++ b/opcode to control bits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrai\Documents\SC8bCPU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5A3259-C6E8-4060-9270-6DA0E14B4B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE840B1-E937-4CD8-9E1F-E14FBF838612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4803" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4806" uniqueCount="193">
   <si>
     <t>Instruction</t>
   </si>
@@ -612,6 +612,21 @@
   <si>
     <t>PC_IN[1:0]</t>
   </si>
+  <si>
+    <t>ALU_Y_SEL[2:0]</t>
+  </si>
+  <si>
+    <t>ALU_X_SEL</t>
+  </si>
+  <si>
+    <t>DMEM_SEL_ADD</t>
+  </si>
+  <si>
+    <t>REG_SEL_IN_A[2:0]</t>
+  </si>
+  <si>
+    <t>REG_SEL_IN_B[1:0]</t>
+  </si>
 </sst>
 </file>
 
@@ -30608,7 +30623,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D896E85-B550-461A-BB89-06512C5EBBCD}">
-  <dimension ref="A1:W62"/>
+  <dimension ref="A1:AB62"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.46484375" style="1" bestFit="1" customWidth="1"/>
@@ -30633,9 +30648,13 @@
     <col min="20" max="20" width="8.9296875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="6" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="6.796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="16.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -30705,8 +30724,23 @@
       <c r="W1" s="1" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="X1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>24</v>
       </c>
@@ -30717,7 +30751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
@@ -30725,7 +30759,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>48</v>
       </c>
@@ -30750,8 +30784,14 @@
       <c r="U4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="X4">
+        <v>1</v>
+      </c>
+      <c r="Y4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>92</v>
       </c>
@@ -30773,8 +30813,14 @@
       <c r="U5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="X5">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>50</v>
       </c>
@@ -30799,8 +30845,11 @@
       <c r="U6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>97</v>
       </c>
@@ -30834,8 +30883,11 @@
       <c r="U7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>138</v>
       </c>
@@ -30863,8 +30915,14 @@
       <c r="U8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="X8">
+        <v>1</v>
+      </c>
+      <c r="Y8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>111</v>
       </c>
@@ -30893,7 +30951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>95</v>
       </c>
@@ -30924,8 +30982,14 @@
       <c r="U10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="X10">
+        <v>1</v>
+      </c>
+      <c r="Y10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>96</v>
       </c>
@@ -30959,8 +31023,14 @@
       <c r="U11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="X11">
+        <v>1</v>
+      </c>
+      <c r="Y11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>139</v>
       </c>
@@ -30983,7 +31053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>140</v>
       </c>
@@ -31014,8 +31084,11 @@
       <c r="W13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AB13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>141</v>
       </c>
@@ -31038,7 +31111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>142</v>
       </c>
@@ -31061,7 +31134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>144</v>
       </c>
@@ -31084,7 +31157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>143</v>
       </c>
@@ -31107,7 +31180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
@@ -31129,8 +31202,11 @@
       <c r="V18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>145</v>
       </c>
@@ -31149,8 +31225,11 @@
       <c r="U19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>146</v>
       </c>
@@ -31169,7 +31248,7 @@
       <c r="M20" t="s">
         <v>153</v>
       </c>
-      <c r="P20" t="s">
+      <c r="Q20" t="s">
         <v>126</v>
       </c>
       <c r="S20">
@@ -31181,8 +31260,14 @@
       <c r="V20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Z20">
+        <v>1</v>
+      </c>
+      <c r="AA20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>147</v>
       </c>
@@ -31201,7 +31286,7 @@
       <c r="M21" t="s">
         <v>153</v>
       </c>
-      <c r="P21" t="s">
+      <c r="Q21" t="s">
         <v>126</v>
       </c>
       <c r="S21">
@@ -31213,8 +31298,14 @@
       <c r="V21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Z21">
+        <v>1</v>
+      </c>
+      <c r="AA21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>148</v>
       </c>
@@ -31233,7 +31324,7 @@
       <c r="M22" t="s">
         <v>153</v>
       </c>
-      <c r="P22" t="s">
+      <c r="Q22" t="s">
         <v>126</v>
       </c>
       <c r="S22">
@@ -31245,8 +31336,14 @@
       <c r="V22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Z22">
+        <v>1</v>
+      </c>
+      <c r="AA22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>149</v>
       </c>
@@ -31259,8 +31356,11 @@
       <c r="D23" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="P23" t="s">
+        <v>153</v>
+      </c>
       <c r="Q23" t="s">
-        <v>153</v>
+        <v>126</v>
       </c>
       <c r="S23">
         <v>3</v>
@@ -31271,8 +31371,11 @@
       <c r="V23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Z23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>150</v>
       </c>
@@ -31285,8 +31388,11 @@
       <c r="D24" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="P24" t="s">
+        <v>153</v>
+      </c>
       <c r="Q24" t="s">
-        <v>153</v>
+        <v>126</v>
       </c>
       <c r="S24">
         <v>1</v>
@@ -31297,8 +31403,11 @@
       <c r="V24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Z24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>151</v>
       </c>
@@ -31311,8 +31420,11 @@
       <c r="D25" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="P25" t="s">
+        <v>153</v>
+      </c>
       <c r="Q25" t="s">
-        <v>153</v>
+        <v>126</v>
       </c>
       <c r="S25">
         <v>0</v>
@@ -31323,8 +31435,11 @@
       <c r="V25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Z25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>107</v>
       </c>
@@ -31352,8 +31467,11 @@
       <c r="U26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>63</v>
       </c>
@@ -31373,7 +31491,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>66</v>
       </c>
@@ -31393,7 +31511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>87</v>
       </c>
@@ -31413,7 +31531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>152</v>
       </c>
@@ -31432,8 +31550,11 @@
       <c r="U30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>101</v>
       </c>
@@ -31479,8 +31600,11 @@
       <c r="U31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>95</v>
       </c>
@@ -31524,7 +31648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>104</v>
       </c>
@@ -31573,8 +31697,11 @@
       <c r="U33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y33">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>96</v>
       </c>
@@ -31621,7 +31748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>106</v>
       </c>
@@ -31667,8 +31794,11 @@
       <c r="U35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>113</v>
       </c>
@@ -31712,7 +31842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>108</v>
       </c>
@@ -31758,8 +31888,11 @@
       <c r="U37">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y37">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>114</v>
       </c>
@@ -31803,7 +31936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>110</v>
       </c>
@@ -31849,8 +31982,11 @@
       <c r="U39">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y39">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
         <v>115</v>
       </c>
@@ -31894,7 +32030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A41" s="1" t="s">
         <v>98</v>
       </c>
@@ -31931,14 +32067,14 @@
       <c r="P41" t="s">
         <v>126</v>
       </c>
-      <c r="Q41" t="s">
-        <v>119</v>
-      </c>
       <c r="U41">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A42" s="1" t="s">
         <v>154</v>
       </c>
@@ -31982,7 +32118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A43" s="1" t="s">
         <v>93</v>
       </c>
@@ -32019,14 +32155,14 @@
       <c r="P43" t="s">
         <v>126</v>
       </c>
-      <c r="Q43" t="s">
-        <v>119</v>
-      </c>
       <c r="U43">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A44" s="1" t="s">
         <v>155</v>
       </c>
@@ -32070,7 +32206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A45" s="1" t="s">
         <v>94</v>
       </c>
@@ -32110,14 +32246,14 @@
       <c r="P45" t="s">
         <v>126</v>
       </c>
-      <c r="Q45" t="s">
-        <v>119</v>
-      </c>
       <c r="U45">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A46" s="1" t="s">
         <v>156</v>
       </c>
@@ -32164,7 +32300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A47" s="1" t="s">
         <v>99</v>
       </c>
@@ -32201,14 +32337,14 @@
       <c r="P47" t="s">
         <v>126</v>
       </c>
-      <c r="Q47" t="s">
-        <v>119</v>
-      </c>
       <c r="U47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="Y47">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="s">
         <v>157</v>
       </c>
@@ -32252,7 +32388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A49" s="1" t="s">
         <v>100</v>
       </c>
@@ -32292,14 +32428,14 @@
       <c r="P49" t="s">
         <v>126</v>
       </c>
-      <c r="Q49" t="s">
-        <v>119</v>
-      </c>
       <c r="U49">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y49">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A50" s="1" t="s">
         <v>158</v>
       </c>
@@ -32346,7 +32482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A51" s="1" t="s">
         <v>159</v>
       </c>
@@ -32401,8 +32537,17 @@
       <c r="V51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y51">
+        <v>4</v>
+      </c>
+      <c r="AA51">
+        <v>6</v>
+      </c>
+      <c r="AB51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A52" s="1" t="s">
         <v>160</v>
       </c>
@@ -32454,8 +32599,14 @@
       <c r="V52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA52">
+        <v>6</v>
+      </c>
+      <c r="AB52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A53" s="1" t="s">
         <v>161</v>
       </c>
@@ -32507,8 +32658,17 @@
       <c r="U53">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y53">
+        <v>4</v>
+      </c>
+      <c r="AA53">
+        <v>6</v>
+      </c>
+      <c r="AB53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A54" s="1" t="s">
         <v>162</v>
       </c>
@@ -32557,8 +32717,14 @@
       <c r="U54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA54">
+        <v>6</v>
+      </c>
+      <c r="AB54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A55" s="1" t="s">
         <v>184</v>
       </c>
@@ -32613,8 +32779,17 @@
       <c r="V55">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y55">
+        <v>4</v>
+      </c>
+      <c r="AA55">
+        <v>7</v>
+      </c>
+      <c r="AB55">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A56" s="1" t="s">
         <v>163</v>
       </c>
@@ -32666,8 +32841,14 @@
       <c r="V56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA56">
+        <v>7</v>
+      </c>
+      <c r="AB56">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A57" s="1" t="s">
         <v>185</v>
       </c>
@@ -32719,8 +32900,17 @@
       <c r="U57">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y57">
+        <v>4</v>
+      </c>
+      <c r="AA57">
+        <v>7</v>
+      </c>
+      <c r="AB57">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A58" s="1" t="s">
         <v>164</v>
       </c>
@@ -32769,8 +32959,14 @@
       <c r="U58">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="AA58">
+        <v>7</v>
+      </c>
+      <c r="AB58">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A59" s="1" t="s">
         <v>167</v>
       </c>
@@ -32798,11 +32994,8 @@
       <c r="U59">
         <v>1</v>
       </c>
-      <c r="W59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.45">
+    </row>
+    <row r="60" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A60" s="1" t="s">
         <v>168</v>
       </c>
@@ -32830,11 +33023,8 @@
       <c r="U60">
         <v>1</v>
       </c>
-      <c r="W60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.45">
+    </row>
+    <row r="61" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A61" s="1" t="s">
         <v>58</v>
       </c>
@@ -32874,8 +33064,11 @@
       <c r="U61">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="Y61">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A62" s="1" t="s">
         <v>169</v>
       </c>
@@ -32908,6 +33101,9 @@
       </c>
       <c r="U62">
         <v>1</v>
+      </c>
+      <c r="Y62">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rewrite most of control unit. Add Memory read enable
</commit_message>
<xml_diff>
--- a/opcode to control bits.xlsx
+++ b/opcode to control bits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrai\Documents\SC8bCPU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE840B1-E937-4CD8-9E1F-E14FBF838612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DFCF7FA-DD6B-4666-B89E-159E25C97183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'v2'!$A$1:$AA$257</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'v3'!$A$1:$AC$257</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'v4'!$A$1:$AA$257</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'v5'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'v5'!$A$1:$AB$62</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -580,12 +580,6 @@
     <t>REG_WE_B</t>
   </si>
   <si>
-    <t>REG_R_ADD_A</t>
-  </si>
-  <si>
-    <t>REG_R_ADD_B</t>
-  </si>
-  <si>
     <t>DMEM_DLEN[1:0]</t>
   </si>
   <si>
@@ -626,6 +620,12 @@
   </si>
   <si>
     <t>REG_SEL_IN_B[1:0]</t>
+  </si>
+  <si>
+    <t>REG_R_ADD_A[4:0]</t>
+  </si>
+  <si>
+    <t>REG_R_ADD_B[4:0]</t>
   </si>
 </sst>
 </file>
@@ -30626,32 +30626,34 @@
   <dimension ref="A1:AB62"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.46484375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.73046875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="2.796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.9296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.19921875" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.46484375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.06640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.59765625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.9296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.59765625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.53125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.06640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.1328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.9296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.59765625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="16.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.9296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.46484375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.53125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.06640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.53125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.53125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.46484375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.265625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.06640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.45">
@@ -30701,16 +30703,16 @@
         <v>174</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>22</v>
@@ -30719,25 +30721,25 @@
         <v>23</v>
       </c>
       <c r="V1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y1" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="Y1" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.45">
@@ -30904,7 +30906,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="P8" t="s">
         <v>119</v>
@@ -30965,7 +30967,7 @@
         <v>119</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -31006,7 +31008,7 @@
         <v>1</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L11">
         <v>1</v>
@@ -31102,7 +31104,7 @@
         <v>126</v>
       </c>
       <c r="T14" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U14">
         <v>1</v>
@@ -31125,7 +31127,7 @@
         <v>126</v>
       </c>
       <c r="T15" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U15">
         <v>1</v>
@@ -31148,7 +31150,7 @@
         <v>126</v>
       </c>
       <c r="T16" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U16">
         <v>1</v>
@@ -31171,7 +31173,7 @@
         <v>126</v>
       </c>
       <c r="T17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U17">
         <v>1</v>
@@ -31327,9 +31329,6 @@
       <c r="Q22" t="s">
         <v>126</v>
       </c>
-      <c r="S22">
-        <v>0</v>
-      </c>
       <c r="U22">
         <v>1</v>
       </c>
@@ -31362,6 +31361,9 @@
       <c r="Q23" t="s">
         <v>126</v>
       </c>
+      <c r="R23">
+        <v>1</v>
+      </c>
       <c r="S23">
         <v>3</v>
       </c>
@@ -31394,6 +31396,9 @@
       <c r="Q24" t="s">
         <v>126</v>
       </c>
+      <c r="R24">
+        <v>1</v>
+      </c>
       <c r="S24">
         <v>1</v>
       </c>
@@ -31426,8 +31431,8 @@
       <c r="Q25" t="s">
         <v>126</v>
       </c>
-      <c r="S25">
-        <v>0</v>
+      <c r="R25">
+        <v>1</v>
       </c>
       <c r="U25">
         <v>1</v>
@@ -31479,7 +31484,7 @@
         <v>133</v>
       </c>
       <c r="T27" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U27">
         <v>1</v>
@@ -31499,7 +31504,7 @@
         <v>28</v>
       </c>
       <c r="T28" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U28">
         <v>1</v>
@@ -31519,7 +31524,7 @@
         <v>29</v>
       </c>
       <c r="T29" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U29">
         <v>1</v>
@@ -31580,7 +31585,7 @@
         <v>123</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L31">
         <v>1</v>
@@ -31630,7 +31635,7 @@
         <v>124</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L32">
         <v>1</v>
@@ -31677,7 +31682,7 @@
         <v>1</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L33">
         <v>1</v>
@@ -31730,7 +31735,7 @@
         <v>1</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L34">
         <v>1</v>
@@ -32508,7 +32513,7 @@
         <v>123</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="L51">
         <v>1</v>
@@ -32573,7 +32578,7 @@
         <v>124</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="L52">
         <v>1</v>
@@ -32632,7 +32637,7 @@
         <v>125</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="L53">
         <v>1</v>
@@ -32694,7 +32699,7 @@
         <v>127</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="L54">
         <v>1</v>
@@ -32726,7 +32731,7 @@
     </row>
     <row r="55" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A55" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>135</v>
@@ -32750,7 +32755,7 @@
         <v>128</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="L55">
         <v>1</v>
@@ -32815,7 +32820,7 @@
         <v>129</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="L56">
         <v>1</v>
@@ -32850,7 +32855,7 @@
     </row>
     <row r="57" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A57" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>135</v>
@@ -32874,7 +32879,7 @@
         <v>130</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="L57">
         <v>1</v>
@@ -32936,7 +32941,7 @@
         <v>131</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="L58">
         <v>1</v>
@@ -32989,7 +32994,7 @@
         <v>126</v>
       </c>
       <c r="T59" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U59">
         <v>1</v>
@@ -33018,7 +33023,7 @@
         <v>126</v>
       </c>
       <c r="T60" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="U60">
         <v>1</v>
@@ -33050,7 +33055,7 @@
         <v>1</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="P61" t="s">
         <v>126</v>
@@ -33107,6 +33112,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AB62" xr:uid="{3D896E85-B550-461A-BB89-06512C5EBBCD}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Complete CPU design and minor additions to Opcode Decoder
</commit_message>
<xml_diff>
--- a/opcode to control bits.xlsx
+++ b/opcode to control bits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrai\Documents\SC8bCPU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DFCF7FA-DD6B-4666-B89E-159E25C97183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A0EF14-09F8-4B2B-8038-2B58766CA6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15" yWindow="15" windowWidth="23025" windowHeight="13665" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4806" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4811" uniqueCount="193">
   <si>
     <t>Instruction</t>
   </si>
@@ -32072,6 +32072,9 @@
       <c r="P41" t="s">
         <v>126</v>
       </c>
+      <c r="Q41" t="s">
+        <v>119</v>
+      </c>
       <c r="U41">
         <v>1</v>
       </c>
@@ -32160,6 +32163,9 @@
       <c r="P43" t="s">
         <v>126</v>
       </c>
+      <c r="Q43" t="s">
+        <v>119</v>
+      </c>
       <c r="U43">
         <v>1</v>
       </c>
@@ -32251,6 +32257,9 @@
       <c r="P45" t="s">
         <v>126</v>
       </c>
+      <c r="Q45" t="s">
+        <v>119</v>
+      </c>
       <c r="U45">
         <v>1</v>
       </c>
@@ -32342,6 +32351,9 @@
       <c r="P47" t="s">
         <v>126</v>
       </c>
+      <c r="Q47" t="s">
+        <v>119</v>
+      </c>
       <c r="U47">
         <v>1</v>
       </c>
@@ -32432,6 +32444,9 @@
       </c>
       <c r="P49" t="s">
         <v>126</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>119</v>
       </c>
       <c r="U49">
         <v>1</v>

</xml_diff>